<commit_message>
UK daily ratings for 2026-05-13
</commit_message>
<xml_diff>
--- a/output/daily_ratings/uk_ratings_2026-05-13.xlsx
+++ b/output/daily_ratings/uk_ratings_2026-05-13.xlsx
@@ -524,34 +524,36 @@
         <v>6</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Up The Anti (IRE)</t>
+          <t>Nordic Glory (IRE)</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J2" t="n">
-        <v>135</v>
+        <v>126</v>
       </c>
       <c r="K2" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
         <v>63.53</v>
       </c>
-      <c r="N2" t="inlineStr"/>
+      <c r="N2" t="n">
+        <v>51.3</v>
+      </c>
       <c r="O2" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>-8.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -580,34 +582,38 @@
         <v>6</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Neptune Legend (IRE)</t>
+          <t>Wedgewood</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J3" t="n">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="K3" t="n">
-        <v>51</v>
-      </c>
-      <c r="L3" t="inlineStr"/>
+        <v>49</v>
+      </c>
+      <c r="L3" t="n">
+        <v>1</v>
+      </c>
       <c r="M3" t="n">
         <v>63.53</v>
       </c>
-      <c r="N3" t="inlineStr"/>
+      <c r="N3" t="n">
+        <v>51.2</v>
+      </c>
       <c r="O3" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>-8.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -636,28 +642,30 @@
         <v>6</v>
       </c>
       <c r="G4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Nordic Glory (IRE)</t>
+          <t>Darkened Edge</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J4" t="n">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="K4" t="n">
-        <v>53</v>
-      </c>
-      <c r="L4" t="inlineStr"/>
+        <v>52</v>
+      </c>
+      <c r="L4" t="n">
+        <v>2.75</v>
+      </c>
       <c r="M4" t="n">
         <v>63.53</v>
       </c>
       <c r="N4" t="n">
-        <v>57.9</v>
+        <v>49.5</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -694,30 +702,30 @@
         <v>6</v>
       </c>
       <c r="G5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Wedgewood</t>
+          <t>Anglesey Lad (IRE)</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J5" t="n">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="K5" t="n">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="L5" t="n">
-        <v>1</v>
+        <v>3.25</v>
       </c>
       <c r="M5" t="n">
         <v>63.53</v>
       </c>
       <c r="N5" t="n">
-        <v>51.2</v>
+        <v>35.8</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -725,7 +733,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="6">
@@ -754,30 +762,30 @@
         <v>6</v>
       </c>
       <c r="G6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Darkened Edge</t>
+          <t>Payforanother Daay</t>
         </is>
       </c>
       <c r="I6" t="n">
         <v>6</v>
       </c>
       <c r="J6" t="n">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="K6" t="n">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="L6" t="n">
-        <v>2.75</v>
+        <v>3.75</v>
       </c>
       <c r="M6" t="n">
         <v>63.53</v>
       </c>
       <c r="N6" t="n">
-        <v>49.5</v>
+        <v>37.3</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -785,7 +793,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -814,15 +822,15 @@
         <v>6</v>
       </c>
       <c r="G7" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Anglesey Lad (IRE)</t>
+          <t>Alyara</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J7" t="n">
         <v>126</v>
@@ -831,13 +839,13 @@
         <v>46</v>
       </c>
       <c r="L7" t="n">
-        <v>3.25</v>
+        <v>5.25</v>
       </c>
       <c r="M7" t="n">
         <v>63.53</v>
       </c>
       <c r="N7" t="n">
-        <v>39.3</v>
+        <v>32.2</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -874,15 +882,15 @@
         <v>6</v>
       </c>
       <c r="G8" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Payforanother Daay</t>
+          <t>Coast</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J8" t="n">
         <v>126</v>
@@ -891,13 +899,13 @@
         <v>46</v>
       </c>
       <c r="L8" t="n">
-        <v>3.75</v>
+        <v>9.25</v>
       </c>
       <c r="M8" t="n">
         <v>63.53</v>
       </c>
       <c r="N8" t="n">
-        <v>37.3</v>
+        <v>17.7</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -933,40 +941,24 @@
       <c r="F9" t="n">
         <v>6</v>
       </c>
-      <c r="G9" t="n">
-        <v>6</v>
-      </c>
+      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Alyara</t>
-        </is>
-      </c>
-      <c r="I9" t="n">
-        <v>8</v>
-      </c>
-      <c r="J9" t="n">
-        <v>126</v>
-      </c>
-      <c r="K9" t="n">
-        <v>46</v>
-      </c>
-      <c r="L9" t="n">
-        <v>5.25</v>
-      </c>
-      <c r="M9" t="n">
-        <v>63.53</v>
-      </c>
-      <c r="N9" t="n">
-        <v>32.2</v>
-      </c>
+          <t>Neptune Legend (IRE)</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="P9" t="n">
-        <v>0</v>
-      </c>
+      <c r="P9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -993,40 +985,24 @@
       <c r="F10" t="n">
         <v>6</v>
       </c>
-      <c r="G10" t="n">
-        <v>7</v>
-      </c>
+      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Coast</t>
-        </is>
-      </c>
-      <c r="I10" t="n">
-        <v>7</v>
-      </c>
-      <c r="J10" t="n">
-        <v>126</v>
-      </c>
-      <c r="K10" t="n">
-        <v>46</v>
-      </c>
-      <c r="L10" t="n">
-        <v>9.25</v>
-      </c>
-      <c r="M10" t="n">
-        <v>63.53</v>
-      </c>
-      <c r="N10" t="n">
-        <v>17.7</v>
-      </c>
+          <t>Up The Anti (IRE)</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="P10" t="n">
-        <v>0</v>
-      </c>
+      <c r="P10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1183,7 +1159,7 @@
         <v>2</v>
       </c>
       <c r="J13" t="n">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="K13" t="n">
         <v>0</v>
@@ -1195,7 +1171,7 @@
         <v>74.06</v>
       </c>
       <c r="N13" t="n">
-        <v>27.5</v>
+        <v>24.4</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1303,7 +1279,7 @@
         <v>2</v>
       </c>
       <c r="J15" t="n">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="K15" t="n">
         <v>0</v>
@@ -1315,7 +1291,7 @@
         <v>74.06</v>
       </c>
       <c r="N15" t="n">
-        <v>22.1</v>
+        <v>15.8</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1710,18 +1686,18 @@
         <v>5</v>
       </c>
       <c r="G22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Sup Of Red (IRE)</t>
+          <t>Foothold (IRE)</t>
         </is>
       </c>
       <c r="I22" t="n">
         <v>3</v>
       </c>
       <c r="J22" t="n">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="K22" t="n">
         <v>62</v>
@@ -1730,14 +1706,16 @@
       <c r="M22" t="n">
         <v>101.97</v>
       </c>
-      <c r="N22" t="inlineStr"/>
+      <c r="N22" t="n">
+        <v>65.3</v>
+      </c>
       <c r="O22" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="P22" t="n">
-        <v>-6.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -1766,34 +1744,38 @@
         <v>5</v>
       </c>
       <c r="G23" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Fizzy Bear (IRE)</t>
+          <t>Phantom Shadow (FR)</t>
         </is>
       </c>
       <c r="I23" t="n">
         <v>3</v>
       </c>
       <c r="J23" t="n">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="K23" t="n">
-        <v>62</v>
-      </c>
-      <c r="L23" t="inlineStr"/>
+        <v>59</v>
+      </c>
+      <c r="L23" t="n">
+        <v>3.5</v>
+      </c>
       <c r="M23" t="n">
         <v>101.97</v>
       </c>
-      <c r="N23" t="inlineStr"/>
+      <c r="N23" t="n">
+        <v>57.1</v>
+      </c>
       <c r="O23" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="P23" t="n">
-        <v>-6.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -1822,28 +1804,30 @@
         <v>5</v>
       </c>
       <c r="G24" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Foothold (IRE)</t>
+          <t>Quilt (IRE)</t>
         </is>
       </c>
       <c r="I24" t="n">
         <v>3</v>
       </c>
       <c r="J24" t="n">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="K24" t="n">
-        <v>62</v>
-      </c>
-      <c r="L24" t="inlineStr"/>
+        <v>68</v>
+      </c>
+      <c r="L24" t="n">
+        <v>8.5</v>
+      </c>
       <c r="M24" t="n">
         <v>101.97</v>
       </c>
       <c r="N24" t="n">
-        <v>70.5</v>
+        <v>54.2</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
@@ -1880,30 +1864,30 @@
         <v>5</v>
       </c>
       <c r="G25" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Phantom Shadow (FR)</t>
+          <t>Just A Gambler (IRE)</t>
         </is>
       </c>
       <c r="I25" t="n">
         <v>3</v>
       </c>
       <c r="J25" t="n">
-        <v>124</v>
+        <v>133</v>
       </c>
       <c r="K25" t="n">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="L25" t="n">
-        <v>3.5</v>
+        <v>10</v>
       </c>
       <c r="M25" t="n">
         <v>101.97</v>
       </c>
       <c r="N25" t="n">
-        <v>57.1</v>
+        <v>51.8</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
@@ -1940,30 +1924,30 @@
         <v>5</v>
       </c>
       <c r="G26" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Quilt (IRE)</t>
+          <t>Halla Bil Zain (IRE)</t>
         </is>
       </c>
       <c r="I26" t="n">
         <v>3</v>
       </c>
       <c r="J26" t="n">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="K26" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="L26" t="n">
-        <v>8.5</v>
+        <v>12.75</v>
       </c>
       <c r="M26" t="n">
         <v>101.97</v>
       </c>
       <c r="N26" t="n">
-        <v>54.2</v>
+        <v>44.9</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
@@ -1999,40 +1983,24 @@
       <c r="F27" t="n">
         <v>5</v>
       </c>
-      <c r="G27" t="n">
-        <v>4</v>
-      </c>
+      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Just A Gambler (IRE)</t>
-        </is>
-      </c>
-      <c r="I27" t="n">
-        <v>3</v>
-      </c>
-      <c r="J27" t="n">
-        <v>133</v>
-      </c>
-      <c r="K27" t="n">
-        <v>68</v>
-      </c>
-      <c r="L27" t="n">
-        <v>10</v>
-      </c>
-      <c r="M27" t="n">
-        <v>101.97</v>
-      </c>
-      <c r="N27" t="n">
-        <v>51.8</v>
-      </c>
+          <t>Fizzy Bear (IRE)</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
       <c r="O27" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="P27" t="n">
-        <v>0</v>
-      </c>
+      <c r="P27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2059,40 +2027,24 @@
       <c r="F28" t="n">
         <v>5</v>
       </c>
-      <c r="G28" t="n">
-        <v>5</v>
-      </c>
+      <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Halla Bil Zain (IRE)</t>
-        </is>
-      </c>
-      <c r="I28" t="n">
-        <v>3</v>
-      </c>
-      <c r="J28" t="n">
-        <v>135</v>
-      </c>
-      <c r="K28" t="n">
-        <v>70</v>
-      </c>
-      <c r="L28" t="n">
-        <v>12.75</v>
-      </c>
-      <c r="M28" t="n">
-        <v>101.97</v>
-      </c>
-      <c r="N28" t="n">
-        <v>44.9</v>
-      </c>
+          <t>Sup Of Red (IRE)</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
       <c r="O28" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="P28" t="n">
-        <v>0</v>
-      </c>
+      <c r="P28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2189,7 +2141,7 @@
         <v>7</v>
       </c>
       <c r="J30" t="n">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="K30" t="n">
         <v>58</v>
@@ -2201,7 +2153,7 @@
         <v>148.41</v>
       </c>
       <c r="N30" t="n">
-        <v>77.59999999999999</v>
+        <v>74.7</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
@@ -2309,7 +2261,7 @@
         <v>4</v>
       </c>
       <c r="J32" t="n">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="K32" t="n">
         <v>52</v>
@@ -2321,7 +2273,7 @@
         <v>148.41</v>
       </c>
       <c r="N32" t="n">
-        <v>66.09999999999999</v>
+        <v>62.2</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
@@ -2369,7 +2321,7 @@
         <v>7</v>
       </c>
       <c r="J33" t="n">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="K33" t="n">
         <v>47</v>
@@ -2381,7 +2333,7 @@
         <v>148.41</v>
       </c>
       <c r="N33" t="n">
-        <v>55.2</v>
+        <v>52.4</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
@@ -2607,7 +2559,7 @@
         <v>3</v>
       </c>
       <c r="J37" t="n">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="K37" t="n">
         <v>54</v>
@@ -2619,7 +2571,7 @@
         <v>130.89</v>
       </c>
       <c r="N37" t="n">
-        <v>69.09999999999999</v>
+        <v>65.8</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
@@ -2747,7 +2699,7 @@
         </is>
       </c>
       <c r="P39" t="n">
-        <v>-1.5</v>
+        <v>-0.5</v>
       </c>
     </row>
     <row r="40">
@@ -2787,7 +2739,7 @@
         <v>3</v>
       </c>
       <c r="J40" t="n">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="K40" t="n">
         <v>51</v>
@@ -2799,7 +2751,7 @@
         <v>130.89</v>
       </c>
       <c r="N40" t="n">
-        <v>58.3</v>
+        <v>56.9</v>
       </c>
       <c r="O40" t="inlineStr">
         <is>
@@ -2807,7 +2759,7 @@
         </is>
       </c>
       <c r="P40" t="n">
-        <v>1</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="41">
@@ -2867,7 +2819,7 @@
         </is>
       </c>
       <c r="P41" t="n">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="42">
@@ -2927,7 +2879,7 @@
         </is>
       </c>
       <c r="P42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43">
@@ -3016,34 +2968,36 @@
         <v>6</v>
       </c>
       <c r="G44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Baynoona (IRE)</t>
+          <t>Man Is King (IRE)</t>
         </is>
       </c>
       <c r="I44" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J44" t="n">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="K44" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="L44" t="inlineStr"/>
       <c r="M44" t="n">
         <v>129.01</v>
       </c>
-      <c r="N44" t="inlineStr"/>
+      <c r="N44" t="n">
+        <v>78</v>
+      </c>
       <c r="O44" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="P44" t="n">
-        <v>-8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
@@ -3072,28 +3026,30 @@
         <v>6</v>
       </c>
       <c r="G45" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>Man Is King (IRE)</t>
+          <t>Galactic Glow (IRE)</t>
         </is>
       </c>
       <c r="I45" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="J45" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="K45" t="n">
-        <v>51</v>
-      </c>
-      <c r="L45" t="inlineStr"/>
+        <v>52</v>
+      </c>
+      <c r="L45" t="n">
+        <v>1.5</v>
+      </c>
       <c r="M45" t="n">
         <v>129.01</v>
       </c>
       <c r="N45" t="n">
-        <v>78</v>
+        <v>74.5</v>
       </c>
       <c r="O45" t="inlineStr">
         <is>
@@ -3130,30 +3086,30 @@
         <v>6</v>
       </c>
       <c r="G46" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>Galactic Glow (IRE)</t>
+          <t>My O My (FR)</t>
         </is>
       </c>
       <c r="I46" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="J46" t="n">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="K46" t="n">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="L46" t="n">
-        <v>1.5</v>
+        <v>5.5</v>
       </c>
       <c r="M46" t="n">
         <v>129.01</v>
       </c>
       <c r="N46" t="n">
-        <v>74.5</v>
+        <v>59.5</v>
       </c>
       <c r="O46" t="inlineStr">
         <is>
@@ -3161,7 +3117,7 @@
         </is>
       </c>
       <c r="P46" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="47">
@@ -3190,30 +3146,30 @@
         <v>6</v>
       </c>
       <c r="G47" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>My O My (FR)</t>
+          <t>Blue Hero (CAN)</t>
         </is>
       </c>
       <c r="I47" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="J47" t="n">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="K47" t="n">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="L47" t="n">
-        <v>5.5</v>
+        <v>5.53</v>
       </c>
       <c r="M47" t="n">
         <v>129.01</v>
       </c>
       <c r="N47" t="n">
-        <v>59.5</v>
+        <v>62.4</v>
       </c>
       <c r="O47" t="inlineStr">
         <is>
@@ -3221,7 +3177,7 @@
         </is>
       </c>
       <c r="P47" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48">
@@ -3250,30 +3206,30 @@
         <v>6</v>
       </c>
       <c r="G48" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>Blue Hero (CAN)</t>
+          <t>Graffiti</t>
         </is>
       </c>
       <c r="I48" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J48" t="n">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="K48" t="n">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="L48" t="n">
-        <v>5.53</v>
+        <v>8.780000000000001</v>
       </c>
       <c r="M48" t="n">
         <v>129.01</v>
       </c>
       <c r="N48" t="n">
-        <v>62.4</v>
+        <v>58.4</v>
       </c>
       <c r="O48" t="inlineStr">
         <is>
@@ -3281,7 +3237,7 @@
         </is>
       </c>
       <c r="P48" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49">
@@ -3310,30 +3266,30 @@
         <v>6</v>
       </c>
       <c r="G49" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Graffiti</t>
+          <t>Ciotog (IRE)</t>
         </is>
       </c>
       <c r="I49" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J49" t="n">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="K49" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="L49" t="n">
-        <v>8.779999999999999</v>
+        <v>10.03</v>
       </c>
       <c r="M49" t="n">
         <v>129.01</v>
       </c>
       <c r="N49" t="n">
-        <v>58.4</v>
+        <v>49.3</v>
       </c>
       <c r="O49" t="inlineStr">
         <is>
@@ -3341,7 +3297,7 @@
         </is>
       </c>
       <c r="P49" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="50">
@@ -3370,38 +3326,38 @@
         <v>6</v>
       </c>
       <c r="G50" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>Ciotog (IRE)</t>
+          <t>Grand Harbour</t>
         </is>
       </c>
       <c r="I50" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="J50" t="n">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="K50" t="n">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="L50" t="n">
-        <v>10.03</v>
+        <v>21.03</v>
       </c>
       <c r="M50" t="n">
         <v>129.01</v>
       </c>
       <c r="N50" t="n">
-        <v>55.6</v>
+        <v>49.6</v>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>low</t>
         </is>
       </c>
       <c r="P50" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51">
@@ -3429,40 +3385,24 @@
       <c r="F51" t="n">
         <v>6</v>
       </c>
-      <c r="G51" t="n">
-        <v>7</v>
-      </c>
+      <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr">
         <is>
-          <t>Grand Harbour</t>
-        </is>
-      </c>
-      <c r="I51" t="n">
-        <v>4</v>
-      </c>
-      <c r="J51" t="n">
-        <v>127</v>
-      </c>
-      <c r="K51" t="n">
-        <v>46</v>
-      </c>
-      <c r="L51" t="n">
-        <v>21.03</v>
-      </c>
-      <c r="M51" t="n">
-        <v>129.01</v>
-      </c>
-      <c r="N51" t="n">
-        <v>49.6</v>
-      </c>
+          <t>Baynoona (IRE)</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr"/>
+      <c r="N51" t="inlineStr"/>
       <c r="O51" t="inlineStr">
         <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="P51" t="n">
-        <v>0</v>
-      </c>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3490,34 +3430,36 @@
         <v>6</v>
       </c>
       <c r="G52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>Hello Cotai (IRE)</t>
+          <t>Kamaway</t>
         </is>
       </c>
       <c r="I52" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J52" t="n">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="K52" t="n">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="L52" t="inlineStr"/>
       <c r="M52" t="n">
         <v>99.37</v>
       </c>
-      <c r="N52" t="inlineStr"/>
+      <c r="N52" t="n">
+        <v>69.7</v>
+      </c>
       <c r="O52" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="P52" t="n">
-        <v>-11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53">
@@ -3546,28 +3488,30 @@
         <v>6</v>
       </c>
       <c r="G53" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>Kamaway</t>
+          <t>Cuban Girl</t>
         </is>
       </c>
       <c r="I53" t="n">
         <v>4</v>
       </c>
       <c r="J53" t="n">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="K53" t="n">
-        <v>60</v>
-      </c>
-      <c r="L53" t="inlineStr"/>
+        <v>62</v>
+      </c>
+      <c r="L53" t="n">
+        <v>3</v>
+      </c>
       <c r="M53" t="n">
         <v>99.37</v>
       </c>
       <c r="N53" t="n">
-        <v>69.7</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="O53" t="inlineStr">
         <is>
@@ -3604,30 +3548,30 @@
         <v>6</v>
       </c>
       <c r="G54" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>Cuban Girl</t>
+          <t>Campani</t>
         </is>
       </c>
       <c r="I54" t="n">
         <v>4</v>
       </c>
       <c r="J54" t="n">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="K54" t="n">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="L54" t="n">
-        <v>3</v>
+        <v>3.75</v>
       </c>
       <c r="M54" t="n">
         <v>99.37</v>
       </c>
       <c r="N54" t="n">
-        <v>64.40000000000001</v>
+        <v>57.9</v>
       </c>
       <c r="O54" t="inlineStr">
         <is>
@@ -3664,30 +3608,30 @@
         <v>6</v>
       </c>
       <c r="G55" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>Campani</t>
+          <t>El Fox</t>
         </is>
       </c>
       <c r="I55" t="n">
         <v>4</v>
       </c>
       <c r="J55" t="n">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="K55" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="L55" t="n">
-        <v>3.75</v>
+        <v>5</v>
       </c>
       <c r="M55" t="n">
         <v>99.37</v>
       </c>
       <c r="N55" t="n">
-        <v>57.9</v>
+        <v>56</v>
       </c>
       <c r="O55" t="inlineStr">
         <is>
@@ -3724,30 +3668,30 @@
         <v>6</v>
       </c>
       <c r="G56" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>El Fox</t>
+          <t>Queen Of Good News</t>
         </is>
       </c>
       <c r="I56" t="n">
         <v>4</v>
       </c>
       <c r="J56" t="n">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="K56" t="n">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="L56" t="n">
-        <v>5</v>
+        <v>9.75</v>
       </c>
       <c r="M56" t="n">
         <v>99.37</v>
       </c>
       <c r="N56" t="n">
-        <v>56</v>
+        <v>50.2</v>
       </c>
       <c r="O56" t="inlineStr">
         <is>
@@ -3784,30 +3728,30 @@
         <v>6</v>
       </c>
       <c r="G57" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Queen Of Good News</t>
+          <t>Siam Fox (IRE)</t>
         </is>
       </c>
       <c r="I57" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="J57" t="n">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="K57" t="n">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="L57" t="n">
-        <v>9.75</v>
+        <v>10.75</v>
       </c>
       <c r="M57" t="n">
         <v>99.37</v>
       </c>
       <c r="N57" t="n">
-        <v>50.2</v>
+        <v>41.5</v>
       </c>
       <c r="O57" t="inlineStr">
         <is>
@@ -3844,30 +3788,30 @@
         <v>6</v>
       </c>
       <c r="G58" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>Siam Fox (IRE)</t>
+          <t>Suitcase Smith</t>
         </is>
       </c>
       <c r="I58" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="J58" t="n">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="K58" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="L58" t="n">
-        <v>10.75</v>
+        <v>15.75</v>
       </c>
       <c r="M58" t="n">
         <v>99.37</v>
       </c>
       <c r="N58" t="n">
-        <v>41.5</v>
+        <v>28</v>
       </c>
       <c r="O58" t="inlineStr">
         <is>
@@ -3875,7 +3819,7 @@
         </is>
       </c>
       <c r="P58" t="n">
-        <v>0</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="59">
@@ -3904,30 +3848,30 @@
         <v>6</v>
       </c>
       <c r="G59" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>Suitcase Smith</t>
+          <t>Gladiadora (IRE)</t>
         </is>
       </c>
       <c r="I59" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J59" t="n">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="K59" t="n">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="L59" t="n">
-        <v>15.75</v>
+        <v>18</v>
       </c>
       <c r="M59" t="n">
         <v>99.37</v>
       </c>
       <c r="N59" t="n">
-        <v>28</v>
+        <v>28.4</v>
       </c>
       <c r="O59" t="inlineStr">
         <is>
@@ -3935,7 +3879,7 @@
         </is>
       </c>
       <c r="P59" t="n">
-        <v>-3</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="60">
@@ -3964,38 +3908,38 @@
         <v>6</v>
       </c>
       <c r="G60" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>Gladiadora (IRE)</t>
+          <t>Volto Di Medusa (IRE)</t>
         </is>
       </c>
       <c r="I60" t="n">
         <v>5</v>
       </c>
       <c r="J60" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="K60" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="L60" t="n">
-        <v>18</v>
+        <v>25.5</v>
       </c>
       <c r="M60" t="n">
         <v>99.37</v>
       </c>
       <c r="N60" t="n">
-        <v>28.4</v>
+        <v>35.3</v>
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>low</t>
         </is>
       </c>
       <c r="P60" t="n">
-        <v>-1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="61">
@@ -4024,30 +3968,30 @@
         <v>6</v>
       </c>
       <c r="G61" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>Volto Di Medusa (IRE)</t>
+          <t>Tonal (FR)</t>
         </is>
       </c>
       <c r="I61" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J61" t="n">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="K61" t="n">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="L61" t="n">
-        <v>25.5</v>
+        <v>25.65</v>
       </c>
       <c r="M61" t="n">
         <v>99.37</v>
       </c>
       <c r="N61" t="n">
-        <v>35.3</v>
+        <v>28.5</v>
       </c>
       <c r="O61" t="inlineStr">
         <is>
@@ -4083,40 +4027,24 @@
       <c r="F62" t="n">
         <v>6</v>
       </c>
-      <c r="G62" t="n">
-        <v>10</v>
-      </c>
+      <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr">
         <is>
-          <t>Tonal (FR)</t>
-        </is>
-      </c>
-      <c r="I62" t="n">
-        <v>6</v>
-      </c>
-      <c r="J62" t="n">
-        <v>132</v>
-      </c>
-      <c r="K62" t="n">
-        <v>62</v>
-      </c>
-      <c r="L62" t="n">
-        <v>25.65</v>
-      </c>
-      <c r="M62" t="n">
-        <v>99.37</v>
-      </c>
-      <c r="N62" t="n">
-        <v>33.6</v>
-      </c>
+          <t>Hello Cotai (IRE)</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr"/>
+      <c r="J62" t="inlineStr"/>
+      <c r="K62" t="inlineStr"/>
+      <c r="L62" t="inlineStr"/>
+      <c r="M62" t="inlineStr"/>
+      <c r="N62" t="inlineStr"/>
       <c r="O62" t="inlineStr">
         <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="P62" t="n">
-        <v>2</v>
-      </c>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -4144,34 +4072,36 @@
         <v>3</v>
       </c>
       <c r="G63" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>Forager</t>
+          <t>Naanas Sparkle</t>
         </is>
       </c>
       <c r="I63" t="n">
         <v>4</v>
       </c>
       <c r="J63" t="n">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="K63" t="n">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="L63" t="inlineStr"/>
       <c r="M63" t="n">
         <v>62.49</v>
       </c>
-      <c r="N63" t="inlineStr"/>
+      <c r="N63" t="n">
+        <v>77.59999999999999</v>
+      </c>
       <c r="O63" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="P63" t="n">
-        <v>-11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="64">
@@ -4200,34 +4130,38 @@
         <v>3</v>
       </c>
       <c r="G64" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>Mesaafi</t>
+          <t>Kinswoman</t>
         </is>
       </c>
       <c r="I64" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J64" t="n">
-        <v>125</v>
+        <v>134</v>
       </c>
       <c r="K64" t="n">
-        <v>79</v>
-      </c>
-      <c r="L64" t="inlineStr"/>
+        <v>88</v>
+      </c>
+      <c r="L64" t="n">
+        <v>0.15</v>
+      </c>
       <c r="M64" t="n">
         <v>62.49</v>
       </c>
-      <c r="N64" t="inlineStr"/>
+      <c r="N64" t="n">
+        <v>76.3</v>
+      </c>
       <c r="O64" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="P64" t="n">
-        <v>-11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="65">
@@ -4256,34 +4190,38 @@
         <v>3</v>
       </c>
       <c r="G65" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>Nogos Dream</t>
+          <t>Alondra</t>
         </is>
       </c>
       <c r="I65" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J65" t="n">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="K65" t="n">
-        <v>79</v>
-      </c>
-      <c r="L65" t="inlineStr"/>
+        <v>76</v>
+      </c>
+      <c r="L65" t="n">
+        <v>2.4</v>
+      </c>
       <c r="M65" t="n">
         <v>62.49</v>
       </c>
-      <c r="N65" t="inlineStr"/>
+      <c r="N65" t="n">
+        <v>60.7</v>
+      </c>
       <c r="O65" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="P65" t="n">
-        <v>-11</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="66">
@@ -4312,34 +4250,38 @@
         <v>3</v>
       </c>
       <c r="G66" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>Cressida Wildes</t>
+          <t>Rocking Ends</t>
         </is>
       </c>
       <c r="I66" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J66" t="n">
-        <v>125</v>
+        <v>135</v>
       </c>
       <c r="K66" t="n">
-        <v>79</v>
-      </c>
-      <c r="L66" t="inlineStr"/>
+        <v>89</v>
+      </c>
+      <c r="L66" t="n">
+        <v>3.15</v>
+      </c>
       <c r="M66" t="n">
         <v>62.49</v>
       </c>
-      <c r="N66" t="inlineStr"/>
+      <c r="N66" t="n">
+        <v>64.59999999999999</v>
+      </c>
       <c r="O66" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="P66" t="n">
-        <v>-11</v>
+        <v>1</v>
       </c>
     </row>
     <row r="67">
@@ -4368,34 +4310,38 @@
         <v>3</v>
       </c>
       <c r="G67" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>Grandlad (IRE)</t>
+          <t>Existent</t>
         </is>
       </c>
       <c r="I67" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J67" t="n">
-        <v>129</v>
+        <v>117</v>
       </c>
       <c r="K67" t="n">
-        <v>83</v>
-      </c>
-      <c r="L67" t="inlineStr"/>
+        <v>76</v>
+      </c>
+      <c r="L67" t="n">
+        <v>3.9</v>
+      </c>
       <c r="M67" t="n">
         <v>62.49</v>
       </c>
-      <c r="N67" t="inlineStr"/>
+      <c r="N67" t="n">
+        <v>48.5</v>
+      </c>
       <c r="O67" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="P67" t="n">
-        <v>-11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="68">
@@ -4424,28 +4370,30 @@
         <v>3</v>
       </c>
       <c r="G68" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>Naanas Sparkle</t>
+          <t>Twilight Fun</t>
         </is>
       </c>
       <c r="I68" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J68" t="n">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="K68" t="n">
-        <v>86</v>
-      </c>
-      <c r="L68" t="inlineStr"/>
+        <v>82</v>
+      </c>
+      <c r="L68" t="n">
+        <v>7.15</v>
+      </c>
       <c r="M68" t="n">
         <v>62.49</v>
       </c>
       <c r="N68" t="n">
-        <v>77.59999999999999</v>
+        <v>48.1</v>
       </c>
       <c r="O68" t="inlineStr">
         <is>
@@ -4482,30 +4430,30 @@
         <v>3</v>
       </c>
       <c r="G69" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>Kinswoman</t>
+          <t>Michaelas Boy (IRE)</t>
         </is>
       </c>
       <c r="I69" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J69" t="n">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="K69" t="n">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="L69" t="n">
-        <v>0.15</v>
+        <v>8.65</v>
       </c>
       <c r="M69" t="n">
         <v>62.49</v>
       </c>
       <c r="N69" t="n">
-        <v>76.3</v>
+        <v>43.8</v>
       </c>
       <c r="O69" t="inlineStr">
         <is>
@@ -4541,40 +4489,24 @@
       <c r="F70" t="n">
         <v>3</v>
       </c>
-      <c r="G70" t="n">
-        <v>3</v>
-      </c>
+      <c r="G70" t="inlineStr"/>
       <c r="H70" t="inlineStr">
         <is>
-          <t>Alondra</t>
-        </is>
-      </c>
-      <c r="I70" t="n">
-        <v>4</v>
-      </c>
-      <c r="J70" t="n">
-        <v>122</v>
-      </c>
-      <c r="K70" t="n">
-        <v>76</v>
-      </c>
-      <c r="L70" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="M70" t="n">
-        <v>62.49</v>
-      </c>
-      <c r="N70" t="n">
-        <v>60.7</v>
-      </c>
+          <t>Mesaafi</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr"/>
+      <c r="J70" t="inlineStr"/>
+      <c r="K70" t="inlineStr"/>
+      <c r="L70" t="inlineStr"/>
+      <c r="M70" t="inlineStr"/>
+      <c r="N70" t="inlineStr"/>
       <c r="O70" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="P70" t="n">
-        <v>-1</v>
-      </c>
+      <c r="P70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -4601,40 +4533,24 @@
       <c r="F71" t="n">
         <v>3</v>
       </c>
-      <c r="G71" t="n">
-        <v>4</v>
-      </c>
+      <c r="G71" t="inlineStr"/>
       <c r="H71" t="inlineStr">
         <is>
-          <t>Rocking Ends</t>
-        </is>
-      </c>
-      <c r="I71" t="n">
-        <v>6</v>
-      </c>
-      <c r="J71" t="n">
-        <v>135</v>
-      </c>
-      <c r="K71" t="n">
-        <v>89</v>
-      </c>
-      <c r="L71" t="n">
-        <v>3.15</v>
-      </c>
-      <c r="M71" t="n">
-        <v>62.49</v>
-      </c>
-      <c r="N71" t="n">
-        <v>64.59999999999999</v>
-      </c>
+          <t>Cressida Wildes</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr"/>
+      <c r="J71" t="inlineStr"/>
+      <c r="K71" t="inlineStr"/>
+      <c r="L71" t="inlineStr"/>
+      <c r="M71" t="inlineStr"/>
+      <c r="N71" t="inlineStr"/>
       <c r="O71" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="P71" t="n">
-        <v>1</v>
-      </c>
+      <c r="P71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -4661,40 +4577,24 @@
       <c r="F72" t="n">
         <v>3</v>
       </c>
-      <c r="G72" t="n">
-        <v>5</v>
-      </c>
+      <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr">
         <is>
-          <t>Existent</t>
-        </is>
-      </c>
-      <c r="I72" t="n">
-        <v>8</v>
-      </c>
-      <c r="J72" t="n">
-        <v>122</v>
-      </c>
-      <c r="K72" t="n">
-        <v>76</v>
-      </c>
-      <c r="L72" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="M72" t="n">
-        <v>62.49</v>
-      </c>
-      <c r="N72" t="n">
-        <v>50.5</v>
-      </c>
+          <t>Almaty Star (IRE)</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr"/>
+      <c r="J72" t="inlineStr"/>
+      <c r="K72" t="inlineStr"/>
+      <c r="L72" t="inlineStr"/>
+      <c r="M72" t="inlineStr"/>
+      <c r="N72" t="inlineStr"/>
       <c r="O72" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="P72" t="n">
-        <v>0</v>
-      </c>
+      <c r="P72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -4721,40 +4621,24 @@
       <c r="F73" t="n">
         <v>3</v>
       </c>
-      <c r="G73" t="n">
-        <v>6</v>
-      </c>
+      <c r="G73" t="inlineStr"/>
       <c r="H73" t="inlineStr">
         <is>
-          <t>Twilight Fun</t>
-        </is>
-      </c>
-      <c r="I73" t="n">
-        <v>6</v>
-      </c>
-      <c r="J73" t="n">
-        <v>128</v>
-      </c>
-      <c r="K73" t="n">
-        <v>82</v>
-      </c>
-      <c r="L73" t="n">
-        <v>7.15</v>
-      </c>
-      <c r="M73" t="n">
-        <v>62.49</v>
-      </c>
-      <c r="N73" t="n">
-        <v>48.1</v>
-      </c>
+          <t>Grandlad (IRE)</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr"/>
+      <c r="J73" t="inlineStr"/>
+      <c r="K73" t="inlineStr"/>
+      <c r="L73" t="inlineStr"/>
+      <c r="M73" t="inlineStr"/>
+      <c r="N73" t="inlineStr"/>
       <c r="O73" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="P73" t="n">
-        <v>0</v>
-      </c>
+      <c r="P73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -4781,40 +4665,24 @@
       <c r="F74" t="n">
         <v>3</v>
       </c>
-      <c r="G74" t="n">
-        <v>7</v>
-      </c>
+      <c r="G74" t="inlineStr"/>
       <c r="H74" t="inlineStr">
         <is>
-          <t>Michaelas Boy (IRE)</t>
-        </is>
-      </c>
-      <c r="I74" t="n">
-        <v>6</v>
-      </c>
-      <c r="J74" t="n">
-        <v>131</v>
-      </c>
-      <c r="K74" t="n">
-        <v>85</v>
-      </c>
-      <c r="L74" t="n">
-        <v>8.65</v>
-      </c>
-      <c r="M74" t="n">
-        <v>62.49</v>
-      </c>
-      <c r="N74" t="n">
-        <v>47.9</v>
-      </c>
+          <t>Forager</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr"/>
+      <c r="J74" t="inlineStr"/>
+      <c r="K74" t="inlineStr"/>
+      <c r="L74" t="inlineStr"/>
+      <c r="M74" t="inlineStr"/>
+      <c r="N74" t="inlineStr"/>
       <c r="O74" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="P74" t="n">
-        <v>0</v>
-      </c>
+      <c r="P74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -4841,40 +4709,24 @@
       <c r="F75" t="n">
         <v>3</v>
       </c>
-      <c r="G75" t="n">
-        <v>8</v>
-      </c>
+      <c r="G75" t="inlineStr"/>
       <c r="H75" t="inlineStr">
         <is>
-          <t>Almaty Star (IRE)</t>
-        </is>
-      </c>
-      <c r="I75" t="n">
-        <v>6</v>
-      </c>
-      <c r="J75" t="n">
-        <v>129</v>
-      </c>
-      <c r="K75" t="n">
-        <v>83</v>
-      </c>
-      <c r="L75" t="n">
-        <v>8.65</v>
-      </c>
-      <c r="M75" t="n">
-        <v>62.49</v>
-      </c>
-      <c r="N75" t="n">
-        <v>44.6</v>
-      </c>
+          <t>Nogos Dream</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr"/>
+      <c r="J75" t="inlineStr"/>
+      <c r="K75" t="inlineStr"/>
+      <c r="L75" t="inlineStr"/>
+      <c r="M75" t="inlineStr"/>
+      <c r="N75" t="inlineStr"/>
       <c r="O75" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="P75" t="n">
-        <v>0</v>
-      </c>
+      <c r="P75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -5331,7 +5183,7 @@
         <v>2</v>
       </c>
       <c r="J83" t="n">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="K83" t="n">
         <v>0</v>
@@ -5343,7 +5195,7 @@
         <v>73.84999999999999</v>
       </c>
       <c r="N83" t="n">
-        <v>10.3</v>
+        <v>7.1</v>
       </c>
       <c r="O83" t="inlineStr">
         <is>
@@ -5380,11 +5232,11 @@
         <v>4</v>
       </c>
       <c r="G84" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>Secret Harvest</t>
+          <t>Creative Queen (USA)</t>
         </is>
       </c>
       <c r="I84" t="n">
@@ -5394,20 +5246,22 @@
         <v>128</v>
       </c>
       <c r="K84" t="n">
-        <v>0</v>
+        <v>71</v>
       </c>
       <c r="L84" t="inlineStr"/>
       <c r="M84" t="n">
         <v>75.3</v>
       </c>
-      <c r="N84" t="inlineStr"/>
+      <c r="N84" t="n">
+        <v>40.3</v>
+      </c>
       <c r="O84" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="P84" t="n">
-        <v>-5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="85">
@@ -5436,11 +5290,11 @@
         <v>4</v>
       </c>
       <c r="G85" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>Creative Queen (USA)</t>
+          <t>Reigning Queen</t>
         </is>
       </c>
       <c r="I85" t="n">
@@ -5450,14 +5304,16 @@
         <v>128</v>
       </c>
       <c r="K85" t="n">
-        <v>71</v>
-      </c>
-      <c r="L85" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="L85" t="n">
+        <v>1.75</v>
+      </c>
       <c r="M85" t="n">
         <v>75.3</v>
       </c>
       <c r="N85" t="n">
-        <v>40.3</v>
+        <v>36.8</v>
       </c>
       <c r="O85" t="inlineStr">
         <is>
@@ -5494,30 +5350,30 @@
         <v>4</v>
       </c>
       <c r="G86" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>Reigning Queen</t>
+          <t>Viviana</t>
         </is>
       </c>
       <c r="I86" t="n">
         <v>3</v>
       </c>
       <c r="J86" t="n">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="K86" t="n">
         <v>0</v>
       </c>
       <c r="L86" t="n">
-        <v>1.75</v>
+        <v>3.5</v>
       </c>
       <c r="M86" t="n">
         <v>75.3</v>
       </c>
       <c r="N86" t="n">
-        <v>36.8</v>
+        <v>27.8</v>
       </c>
       <c r="O86" t="inlineStr">
         <is>
@@ -5554,11 +5410,11 @@
         <v>4</v>
       </c>
       <c r="G87" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>Viviana</t>
+          <t>Butterfly Beach (IRE)</t>
         </is>
       </c>
       <c r="I87" t="n">
@@ -5568,16 +5424,16 @@
         <v>128</v>
       </c>
       <c r="K87" t="n">
-        <v>0</v>
+        <v>74</v>
       </c>
       <c r="L87" t="n">
-        <v>3.5</v>
+        <v>12</v>
       </c>
       <c r="M87" t="n">
         <v>75.3</v>
       </c>
       <c r="N87" t="n">
-        <v>30.4</v>
+        <v>5.2</v>
       </c>
       <c r="O87" t="inlineStr">
         <is>
@@ -5613,40 +5469,24 @@
       <c r="F88" t="n">
         <v>4</v>
       </c>
-      <c r="G88" t="n">
-        <v>4</v>
-      </c>
+      <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr">
         <is>
-          <t>Butterfly Beach (IRE)</t>
-        </is>
-      </c>
-      <c r="I88" t="n">
-        <v>3</v>
-      </c>
-      <c r="J88" t="n">
-        <v>128</v>
-      </c>
-      <c r="K88" t="n">
-        <v>74</v>
-      </c>
-      <c r="L88" t="n">
-        <v>12</v>
-      </c>
-      <c r="M88" t="n">
-        <v>75.3</v>
-      </c>
-      <c r="N88" t="n">
-        <v>5.2</v>
-      </c>
+          <t>Secret Harvest</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr"/>
+      <c r="J88" t="inlineStr"/>
+      <c r="K88" t="inlineStr"/>
+      <c r="L88" t="inlineStr"/>
+      <c r="M88" t="inlineStr"/>
+      <c r="N88" t="inlineStr"/>
       <c r="O88" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="P88" t="n">
-        <v>0</v>
-      </c>
+      <c r="P88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -5674,34 +5514,36 @@
         <v>4</v>
       </c>
       <c r="G89" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>Fifty Nifty (IRE)</t>
+          <t>Beagle Bay (FR)</t>
         </is>
       </c>
       <c r="I89" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J89" t="n">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="K89" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="L89" t="inlineStr"/>
       <c r="M89" t="n">
         <v>86.95</v>
       </c>
-      <c r="N89" t="inlineStr"/>
+      <c r="N89" t="n">
+        <v>60.2</v>
+      </c>
       <c r="O89" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="P89" t="n">
-        <v>-8.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="90">
@@ -5730,34 +5572,38 @@
         <v>4</v>
       </c>
       <c r="G90" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>Believe The Storm (IRE)</t>
+          <t>Berry Clever</t>
         </is>
       </c>
       <c r="I90" t="n">
         <v>5</v>
       </c>
       <c r="J90" t="n">
-        <v>136</v>
+        <v>122</v>
       </c>
       <c r="K90" t="n">
-        <v>81</v>
-      </c>
-      <c r="L90" t="inlineStr"/>
+        <v>70</v>
+      </c>
+      <c r="L90" t="n">
+        <v>4</v>
+      </c>
       <c r="M90" t="n">
         <v>86.95</v>
       </c>
-      <c r="N90" t="inlineStr"/>
+      <c r="N90" t="n">
+        <v>40.6</v>
+      </c>
       <c r="O90" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="P90" t="n">
-        <v>-8.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="91">
@@ -5786,28 +5632,30 @@
         <v>4</v>
       </c>
       <c r="G91" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>Beagle Bay (FR)</t>
+          <t>Physique (IRE)</t>
         </is>
       </c>
       <c r="I91" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J91" t="n">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="K91" t="n">
-        <v>80</v>
-      </c>
-      <c r="L91" t="inlineStr"/>
+        <v>79</v>
+      </c>
+      <c r="L91" t="n">
+        <v>9</v>
+      </c>
       <c r="M91" t="n">
         <v>86.95</v>
       </c>
       <c r="N91" t="n">
-        <v>60.2</v>
+        <v>39.2</v>
       </c>
       <c r="O91" t="inlineStr">
         <is>
@@ -5844,30 +5692,30 @@
         <v>4</v>
       </c>
       <c r="G92" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>Berry Clever</t>
+          <t>Anthropologist</t>
         </is>
       </c>
       <c r="I92" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J92" t="n">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="K92" t="n">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="L92" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="M92" t="n">
         <v>86.95</v>
       </c>
       <c r="N92" t="n">
-        <v>43.3</v>
+        <v>26.9</v>
       </c>
       <c r="O92" t="inlineStr">
         <is>
@@ -5904,30 +5752,30 @@
         <v>4</v>
       </c>
       <c r="G93" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>Physique (IRE)</t>
+          <t>Noble Guest</t>
         </is>
       </c>
       <c r="I93" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J93" t="n">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="K93" t="n">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="L93" t="n">
-        <v>9</v>
+        <v>14.75</v>
       </c>
       <c r="M93" t="n">
         <v>86.95</v>
       </c>
       <c r="N93" t="n">
-        <v>39.2</v>
+        <v>22.9</v>
       </c>
       <c r="O93" t="inlineStr">
         <is>
@@ -5964,34 +5812,34 @@
         <v>4</v>
       </c>
       <c r="G94" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>Anthropologist</t>
+          <t>Potomac River</t>
         </is>
       </c>
       <c r="I94" t="n">
         <v>4</v>
       </c>
       <c r="J94" t="n">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="K94" t="n">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="L94" t="n">
-        <v>14</v>
+        <v>21.25</v>
       </c>
       <c r="M94" t="n">
         <v>86.95</v>
       </c>
       <c r="N94" t="n">
-        <v>26.9</v>
+        <v>22</v>
       </c>
       <c r="O94" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>low</t>
         </is>
       </c>
       <c r="P94" t="n">
@@ -6024,34 +5872,34 @@
         <v>4</v>
       </c>
       <c r="G95" t="n">
+        <v>7</v>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>Shimmering Spin (USA)</t>
+        </is>
+      </c>
+      <c r="I95" t="n">
         <v>5</v>
       </c>
-      <c r="H95" t="inlineStr">
-        <is>
-          <t>Noble Guest</t>
-        </is>
-      </c>
-      <c r="I95" t="n">
-        <v>4</v>
-      </c>
       <c r="J95" t="n">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="K95" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="L95" t="n">
-        <v>14.75</v>
+        <v>22.75</v>
       </c>
       <c r="M95" t="n">
         <v>86.95</v>
       </c>
       <c r="N95" t="n">
-        <v>22.9</v>
+        <v>13</v>
       </c>
       <c r="O95" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>low</t>
         </is>
       </c>
       <c r="P95" t="n">
@@ -6083,40 +5931,24 @@
       <c r="F96" t="n">
         <v>4</v>
       </c>
-      <c r="G96" t="n">
-        <v>6</v>
-      </c>
+      <c r="G96" t="inlineStr"/>
       <c r="H96" t="inlineStr">
         <is>
-          <t>Potomac River</t>
-        </is>
-      </c>
-      <c r="I96" t="n">
-        <v>4</v>
-      </c>
-      <c r="J96" t="n">
-        <v>132</v>
-      </c>
-      <c r="K96" t="n">
-        <v>77</v>
-      </c>
-      <c r="L96" t="n">
-        <v>21.25</v>
-      </c>
-      <c r="M96" t="n">
-        <v>86.95</v>
-      </c>
-      <c r="N96" t="n">
-        <v>22</v>
-      </c>
+          <t>Believe The Storm (IRE)</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr"/>
+      <c r="J96" t="inlineStr"/>
+      <c r="K96" t="inlineStr"/>
+      <c r="L96" t="inlineStr"/>
+      <c r="M96" t="inlineStr"/>
+      <c r="N96" t="inlineStr"/>
       <c r="O96" t="inlineStr">
         <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="P96" t="n">
-        <v>0</v>
-      </c>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -6143,40 +5975,24 @@
       <c r="F97" t="n">
         <v>4</v>
       </c>
-      <c r="G97" t="n">
-        <v>7</v>
-      </c>
+      <c r="G97" t="inlineStr"/>
       <c r="H97" t="inlineStr">
         <is>
-          <t>Shimmering Spin (USA)</t>
-        </is>
-      </c>
-      <c r="I97" t="n">
-        <v>5</v>
-      </c>
-      <c r="J97" t="n">
-        <v>128</v>
-      </c>
-      <c r="K97" t="n">
-        <v>73</v>
-      </c>
-      <c r="L97" t="n">
-        <v>22.75</v>
-      </c>
-      <c r="M97" t="n">
-        <v>86.95</v>
-      </c>
-      <c r="N97" t="n">
-        <v>13</v>
-      </c>
+          <t>Fifty Nifty (IRE)</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr"/>
+      <c r="J97" t="inlineStr"/>
+      <c r="K97" t="inlineStr"/>
+      <c r="L97" t="inlineStr"/>
+      <c r="M97" t="inlineStr"/>
+      <c r="N97" t="inlineStr"/>
       <c r="O97" t="inlineStr">
         <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="P97" t="n">
-        <v>0</v>
-      </c>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -6204,34 +6020,36 @@
         <v>5</v>
       </c>
       <c r="G98" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>Victor Cee</t>
+          <t>U S S Charleston</t>
         </is>
       </c>
       <c r="I98" t="n">
         <v>3</v>
       </c>
       <c r="J98" t="n">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="K98" t="n">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="L98" t="inlineStr"/>
       <c r="M98" t="n">
         <v>62.93</v>
       </c>
-      <c r="N98" t="inlineStr"/>
+      <c r="N98" t="n">
+        <v>71.59999999999999</v>
+      </c>
       <c r="O98" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="P98" t="n">
-        <v>-6.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="99">
@@ -6260,34 +6078,38 @@
         <v>5</v>
       </c>
       <c r="G99" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>London Is Blue</t>
+          <t>Koffee And Kale</t>
         </is>
       </c>
       <c r="I99" t="n">
         <v>3</v>
       </c>
       <c r="J99" t="n">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="K99" t="n">
-        <v>71</v>
-      </c>
-      <c r="L99" t="inlineStr"/>
+        <v>73</v>
+      </c>
+      <c r="L99" t="n">
+        <v>4</v>
+      </c>
       <c r="M99" t="n">
         <v>62.93</v>
       </c>
-      <c r="N99" t="inlineStr"/>
+      <c r="N99" t="n">
+        <v>64.40000000000001</v>
+      </c>
       <c r="O99" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="P99" t="n">
-        <v>-6.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="100">
@@ -6316,28 +6138,30 @@
         <v>5</v>
       </c>
       <c r="G100" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>U S S Charleston</t>
+          <t>Staniel Cay (IRE)</t>
         </is>
       </c>
       <c r="I100" t="n">
         <v>3</v>
       </c>
       <c r="J100" t="n">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="K100" t="n">
-        <v>71</v>
-      </c>
-      <c r="L100" t="inlineStr"/>
+        <v>67</v>
+      </c>
+      <c r="L100" t="n">
+        <v>5.25</v>
+      </c>
       <c r="M100" t="n">
         <v>62.93</v>
       </c>
       <c r="N100" t="n">
-        <v>73.2</v>
+        <v>54.6</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
@@ -6374,11 +6198,11 @@
         <v>5</v>
       </c>
       <c r="G101" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>Koffee And Kale</t>
+          <t>Grey Horizon</t>
         </is>
       </c>
       <c r="I101" t="n">
@@ -6391,13 +6215,13 @@
         <v>73</v>
       </c>
       <c r="L101" t="n">
-        <v>4</v>
+        <v>8.5</v>
       </c>
       <c r="M101" t="n">
         <v>62.93</v>
       </c>
       <c r="N101" t="n">
-        <v>64.40000000000001</v>
+        <v>50.8</v>
       </c>
       <c r="O101" t="inlineStr">
         <is>
@@ -6434,30 +6258,30 @@
         <v>5</v>
       </c>
       <c r="G102" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>Staniel Cay (IRE)</t>
+          <t>Loleeta</t>
         </is>
       </c>
       <c r="I102" t="n">
         <v>3</v>
       </c>
       <c r="J102" t="n">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="K102" t="n">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="L102" t="n">
-        <v>5.25</v>
+        <v>14.5</v>
       </c>
       <c r="M102" t="n">
         <v>62.93</v>
       </c>
       <c r="N102" t="n">
-        <v>54.6</v>
+        <v>26</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
@@ -6493,40 +6317,24 @@
       <c r="F103" t="n">
         <v>5</v>
       </c>
-      <c r="G103" t="n">
-        <v>4</v>
-      </c>
+      <c r="G103" t="inlineStr"/>
       <c r="H103" t="inlineStr">
         <is>
-          <t>Grey Horizon</t>
-        </is>
-      </c>
-      <c r="I103" t="n">
-        <v>3</v>
-      </c>
-      <c r="J103" t="n">
-        <v>135</v>
-      </c>
-      <c r="K103" t="n">
-        <v>73</v>
-      </c>
-      <c r="L103" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="M103" t="n">
-        <v>62.93</v>
-      </c>
-      <c r="N103" t="n">
-        <v>50.8</v>
-      </c>
+          <t>Victor Cee</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr"/>
+      <c r="J103" t="inlineStr"/>
+      <c r="K103" t="inlineStr"/>
+      <c r="L103" t="inlineStr"/>
+      <c r="M103" t="inlineStr"/>
+      <c r="N103" t="inlineStr"/>
       <c r="O103" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="P103" t="n">
-        <v>0</v>
-      </c>
+      <c r="P103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -6553,40 +6361,24 @@
       <c r="F104" t="n">
         <v>5</v>
       </c>
-      <c r="G104" t="n">
-        <v>5</v>
-      </c>
+      <c r="G104" t="inlineStr"/>
       <c r="H104" t="inlineStr">
         <is>
-          <t>Loleeta</t>
-        </is>
-      </c>
-      <c r="I104" t="n">
-        <v>3</v>
-      </c>
-      <c r="J104" t="n">
-        <v>134</v>
-      </c>
-      <c r="K104" t="n">
-        <v>72</v>
-      </c>
-      <c r="L104" t="n">
-        <v>14.5</v>
-      </c>
-      <c r="M104" t="n">
-        <v>62.93</v>
-      </c>
-      <c r="N104" t="n">
-        <v>32.1</v>
-      </c>
+          <t>London Is Blue</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr"/>
+      <c r="J104" t="inlineStr"/>
+      <c r="K104" t="inlineStr"/>
+      <c r="L104" t="inlineStr"/>
+      <c r="M104" t="inlineStr"/>
+      <c r="N104" t="inlineStr"/>
       <c r="O104" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="P104" t="n">
-        <v>0</v>
-      </c>
+      <c r="P104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -6972,15 +6764,15 @@
         <v>2</v>
       </c>
       <c r="G111" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>Fireblade</t>
+          <t>Klassleader</t>
         </is>
       </c>
       <c r="I111" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J111" t="n">
         <v>125</v>
@@ -6992,14 +6784,16 @@
       <c r="M111" t="n">
         <v>154.26</v>
       </c>
-      <c r="N111" t="inlineStr"/>
+      <c r="N111" t="n">
+        <v>65.09999999999999</v>
+      </c>
       <c r="O111" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="P111" t="n">
-        <v>-11</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="112">
@@ -7028,28 +6822,30 @@
         <v>2</v>
       </c>
       <c r="G112" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>Klassleader</t>
+          <t>Sing Us A Song (IRE)</t>
         </is>
       </c>
       <c r="I112" t="n">
         <v>4</v>
       </c>
       <c r="J112" t="n">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="K112" t="n">
-        <v>90</v>
-      </c>
-      <c r="L112" t="inlineStr"/>
+        <v>95</v>
+      </c>
+      <c r="L112" t="n">
+        <v>2.75</v>
+      </c>
       <c r="M112" t="n">
         <v>154.26</v>
       </c>
       <c r="N112" t="n">
-        <v>65.09999999999999</v>
+        <v>65.5</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -7057,7 +6853,7 @@
         </is>
       </c>
       <c r="P112" t="n">
-        <v>-2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="113">
@@ -7086,30 +6882,30 @@
         <v>2</v>
       </c>
       <c r="G113" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>Sing Us A Song (IRE)</t>
+          <t>Plage De Havre</t>
         </is>
       </c>
       <c r="I113" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J113" t="n">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="K113" t="n">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="L113" t="n">
-        <v>2.75</v>
+        <v>5.25</v>
       </c>
       <c r="M113" t="n">
         <v>154.26</v>
       </c>
       <c r="N113" t="n">
-        <v>65.5</v>
+        <v>65.3</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -7146,30 +6942,30 @@
         <v>2</v>
       </c>
       <c r="G114" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>Plage De Havre</t>
+          <t>Saint Etienne</t>
         </is>
       </c>
       <c r="I114" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J114" t="n">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="K114" t="n">
-        <v>103</v>
+        <v>94</v>
       </c>
       <c r="L114" t="n">
-        <v>5.25</v>
+        <v>6.25</v>
       </c>
       <c r="M114" t="n">
         <v>154.26</v>
       </c>
       <c r="N114" t="n">
-        <v>65.3</v>
+        <v>57</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
@@ -7177,7 +6973,7 @@
         </is>
       </c>
       <c r="P114" t="n">
-        <v>1</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="115">
@@ -7206,30 +7002,30 @@
         <v>2</v>
       </c>
       <c r="G115" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>Saint Etienne</t>
+          <t>Dark Moon Rising (IRE)</t>
         </is>
       </c>
       <c r="I115" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J115" t="n">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="K115" t="n">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="L115" t="n">
-        <v>6.25</v>
+        <v>8</v>
       </c>
       <c r="M115" t="n">
         <v>154.26</v>
       </c>
       <c r="N115" t="n">
-        <v>57</v>
+        <v>49.8</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
@@ -7237,7 +7033,7 @@
         </is>
       </c>
       <c r="P115" t="n">
-        <v>-2</v>
+        <v>-4</v>
       </c>
     </row>
     <row r="116">
@@ -7266,30 +7062,30 @@
         <v>2</v>
       </c>
       <c r="G116" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>Dark Moon Rising (IRE)</t>
+          <t>Paddy The Squire</t>
         </is>
       </c>
       <c r="I116" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J116" t="n">
-        <v>121</v>
+        <v>136</v>
       </c>
       <c r="K116" t="n">
-        <v>86</v>
+        <v>101</v>
       </c>
       <c r="L116" t="n">
-        <v>8</v>
+        <v>8.15</v>
       </c>
       <c r="M116" t="n">
         <v>154.26</v>
       </c>
       <c r="N116" t="n">
-        <v>49.8</v>
+        <v>60.5</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
@@ -7297,7 +7093,7 @@
         </is>
       </c>
       <c r="P116" t="n">
-        <v>-4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="117">
@@ -7326,11 +7122,11 @@
         <v>2</v>
       </c>
       <c r="G117" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>Paddy The Squire</t>
+          <t>Stressfree (FR)</t>
         </is>
       </c>
       <c r="I117" t="n">
@@ -7343,13 +7139,13 @@
         <v>101</v>
       </c>
       <c r="L117" t="n">
-        <v>8.15</v>
+        <v>9.9</v>
       </c>
       <c r="M117" t="n">
         <v>154.26</v>
       </c>
       <c r="N117" t="n">
-        <v>60.5</v>
+        <v>58.4</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -7386,30 +7182,30 @@
         <v>2</v>
       </c>
       <c r="G118" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>Stressfree (FR)</t>
+          <t>Prince Of The Seas (IRE)</t>
         </is>
       </c>
       <c r="I118" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J118" t="n">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="K118" t="n">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="L118" t="n">
-        <v>9.9</v>
+        <v>18.9</v>
       </c>
       <c r="M118" t="n">
         <v>154.26</v>
       </c>
       <c r="N118" t="n">
-        <v>58.4</v>
+        <v>33.7</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
@@ -7417,7 +7213,7 @@
         </is>
       </c>
       <c r="P118" t="n">
-        <v>2</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="119">
@@ -7446,38 +7242,38 @@
         <v>2</v>
       </c>
       <c r="G119" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>Prince Of The Seas (IRE)</t>
+          <t>Will Scarlet</t>
         </is>
       </c>
       <c r="I119" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J119" t="n">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="K119" t="n">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="L119" t="n">
-        <v>18.9</v>
+        <v>20.9</v>
       </c>
       <c r="M119" t="n">
         <v>154.26</v>
       </c>
       <c r="N119" t="n">
-        <v>33.7</v>
+        <v>52.7</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>low</t>
         </is>
       </c>
       <c r="P119" t="n">
-        <v>-2</v>
+        <v>2</v>
       </c>
     </row>
     <row r="120">
@@ -7506,30 +7302,30 @@
         <v>2</v>
       </c>
       <c r="G120" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>Will Scarlet</t>
+          <t>Kings Code</t>
         </is>
       </c>
       <c r="I120" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J120" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="K120" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="L120" t="n">
-        <v>20.9</v>
+        <v>23.65</v>
       </c>
       <c r="M120" t="n">
         <v>154.26</v>
       </c>
       <c r="N120" t="n">
-        <v>52.7</v>
+        <v>50.8</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
@@ -7565,40 +7361,24 @@
       <c r="F121" t="n">
         <v>2</v>
       </c>
-      <c r="G121" t="n">
-        <v>10</v>
-      </c>
+      <c r="G121" t="inlineStr"/>
       <c r="H121" t="inlineStr">
         <is>
-          <t>Kings Code</t>
-        </is>
-      </c>
-      <c r="I121" t="n">
-        <v>6</v>
-      </c>
-      <c r="J121" t="n">
-        <v>134</v>
-      </c>
-      <c r="K121" t="n">
-        <v>99</v>
-      </c>
-      <c r="L121" t="n">
-        <v>23.65</v>
-      </c>
-      <c r="M121" t="n">
-        <v>154.26</v>
-      </c>
-      <c r="N121" t="n">
-        <v>50.8</v>
-      </c>
+          <t>Fireblade</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr"/>
+      <c r="J121" t="inlineStr"/>
+      <c r="K121" t="inlineStr"/>
+      <c r="L121" t="inlineStr"/>
+      <c r="M121" t="inlineStr"/>
+      <c r="N121" t="inlineStr"/>
       <c r="O121" t="inlineStr">
         <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="P121" t="n">
-        <v>2</v>
-      </c>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -9722,11 +9502,11 @@
         <v>1</v>
       </c>
       <c r="G157" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>Della Pace</t>
+          <t>Legacy Link</t>
         </is>
       </c>
       <c r="I157" t="n">
@@ -9736,20 +9516,22 @@
         <v>128</v>
       </c>
       <c r="K157" t="n">
-        <v>82</v>
+        <v>105</v>
       </c>
       <c r="L157" t="inlineStr"/>
       <c r="M157" t="n">
         <v>131.15</v>
       </c>
-      <c r="N157" t="inlineStr"/>
+      <c r="N157" t="n">
+        <v>73</v>
+      </c>
       <c r="O157" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="P157" t="n">
-        <v>-6</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="158">
@@ -9778,11 +9560,11 @@
         <v>1</v>
       </c>
       <c r="G158" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>Legacy Link</t>
+          <t>Felicitas</t>
         </is>
       </c>
       <c r="I158" t="n">
@@ -9792,14 +9574,16 @@
         <v>128</v>
       </c>
       <c r="K158" t="n">
-        <v>105</v>
-      </c>
-      <c r="L158" t="inlineStr"/>
+        <v>96</v>
+      </c>
+      <c r="L158" t="n">
+        <v>0.75</v>
+      </c>
       <c r="M158" t="n">
         <v>131.15</v>
       </c>
       <c r="N158" t="n">
-        <v>73</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="O158" t="inlineStr">
         <is>
@@ -9807,7 +9591,7 @@
         </is>
       </c>
       <c r="P158" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="159">
@@ -9836,11 +9620,11 @@
         <v>1</v>
       </c>
       <c r="G159" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>Felicitas</t>
+          <t>K Sarra</t>
         </is>
       </c>
       <c r="I159" t="n">
@@ -9850,16 +9634,16 @@
         <v>128</v>
       </c>
       <c r="K159" t="n">
-        <v>96</v>
+        <v>82</v>
       </c>
       <c r="L159" t="n">
-        <v>0.75</v>
+        <v>2.25</v>
       </c>
       <c r="M159" t="n">
         <v>131.15</v>
       </c>
       <c r="N159" t="n">
-        <v>73.40000000000001</v>
+        <v>72</v>
       </c>
       <c r="O159" t="inlineStr">
         <is>
@@ -9867,7 +9651,7 @@
         </is>
       </c>
       <c r="P159" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="160">
@@ -9896,11 +9680,11 @@
         <v>1</v>
       </c>
       <c r="G160" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>K Sarra</t>
+          <t>Moments Of Joy (USA)</t>
         </is>
       </c>
       <c r="I160" t="n">
@@ -9910,16 +9694,16 @@
         <v>128</v>
       </c>
       <c r="K160" t="n">
-        <v>82</v>
+        <v>101</v>
       </c>
       <c r="L160" t="n">
-        <v>2.25</v>
+        <v>9.25</v>
       </c>
       <c r="M160" t="n">
         <v>131.15</v>
       </c>
       <c r="N160" t="n">
-        <v>72</v>
+        <v>64.7</v>
       </c>
       <c r="O160" t="inlineStr">
         <is>
@@ -9956,11 +9740,11 @@
         <v>1</v>
       </c>
       <c r="G161" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>Moments Of Joy (USA)</t>
+          <t>Sea The Storm (FR)</t>
         </is>
       </c>
       <c r="I161" t="n">
@@ -9970,16 +9754,16 @@
         <v>128</v>
       </c>
       <c r="K161" t="n">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="L161" t="n">
-        <v>9.25</v>
+        <v>14.25</v>
       </c>
       <c r="M161" t="n">
         <v>131.15</v>
       </c>
       <c r="N161" t="n">
-        <v>64.7</v>
+        <v>57.1</v>
       </c>
       <c r="O161" t="inlineStr">
         <is>
@@ -10015,40 +9799,24 @@
       <c r="F162" t="n">
         <v>1</v>
       </c>
-      <c r="G162" t="n">
-        <v>5</v>
-      </c>
+      <c r="G162" t="inlineStr"/>
       <c r="H162" t="inlineStr">
         <is>
-          <t>Sea The Storm (FR)</t>
-        </is>
-      </c>
-      <c r="I162" t="n">
-        <v>3</v>
-      </c>
-      <c r="J162" t="n">
-        <v>128</v>
-      </c>
-      <c r="K162" t="n">
-        <v>96</v>
-      </c>
-      <c r="L162" t="n">
-        <v>14.25</v>
-      </c>
-      <c r="M162" t="n">
-        <v>131.15</v>
-      </c>
-      <c r="N162" t="n">
-        <v>57.1</v>
-      </c>
+          <t>Della Pace</t>
+        </is>
+      </c>
+      <c r="I162" t="inlineStr"/>
+      <c r="J162" t="inlineStr"/>
+      <c r="K162" t="inlineStr"/>
+      <c r="L162" t="inlineStr"/>
+      <c r="M162" t="inlineStr"/>
+      <c r="N162" t="inlineStr"/>
       <c r="O162" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="P162" t="n">
-        <v>0</v>
-      </c>
+      <c r="P162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -10076,34 +9844,36 @@
         <v>3</v>
       </c>
       <c r="G163" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>Cotai Lights (IRE)</t>
+          <t>Startled (IRE)</t>
         </is>
       </c>
       <c r="I163" t="n">
         <v>3</v>
       </c>
       <c r="J163" t="n">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="K163" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="L163" t="inlineStr"/>
       <c r="M163" t="n">
         <v>87.08</v>
       </c>
-      <c r="N163" t="inlineStr"/>
+      <c r="N163" t="n">
+        <v>64.7</v>
+      </c>
       <c r="O163" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="P163" t="n">
-        <v>-15.5</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="164">
@@ -10132,34 +9902,38 @@
         <v>3</v>
       </c>
       <c r="G164" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>Passing Thought</t>
+          <t>Daydreama</t>
         </is>
       </c>
       <c r="I164" t="n">
         <v>3</v>
       </c>
       <c r="J164" t="n">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="K164" t="n">
-        <v>85</v>
-      </c>
-      <c r="L164" t="inlineStr"/>
+        <v>88</v>
+      </c>
+      <c r="L164" t="n">
+        <v>1.5</v>
+      </c>
       <c r="M164" t="n">
         <v>87.08</v>
       </c>
-      <c r="N164" t="inlineStr"/>
+      <c r="N164" t="n">
+        <v>67.59999999999999</v>
+      </c>
       <c r="O164" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="P164" t="n">
-        <v>-15.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="165">
@@ -10188,11 +9962,11 @@
         <v>3</v>
       </c>
       <c r="G165" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>Startled (IRE)</t>
+          <t>The Resdev Scholar (IRE)</t>
         </is>
       </c>
       <c r="I165" t="n">
@@ -10204,12 +9978,14 @@
       <c r="K165" t="n">
         <v>78</v>
       </c>
-      <c r="L165" t="inlineStr"/>
+      <c r="L165" t="n">
+        <v>2</v>
+      </c>
       <c r="M165" t="n">
         <v>87.08</v>
       </c>
       <c r="N165" t="n">
-        <v>64.7</v>
+        <v>58.9</v>
       </c>
       <c r="O165" t="inlineStr">
         <is>
@@ -10217,7 +9993,7 @@
         </is>
       </c>
       <c r="P165" t="n">
-        <v>-3</v>
+        <v>-4</v>
       </c>
     </row>
     <row r="166">
@@ -10246,30 +10022,30 @@
         <v>3</v>
       </c>
       <c r="G166" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>Daydreama</t>
+          <t>Gold Queen Kindly (IRE)</t>
         </is>
       </c>
       <c r="I166" t="n">
         <v>3</v>
       </c>
       <c r="J166" t="n">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="K166" t="n">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="L166" t="n">
-        <v>1.5</v>
+        <v>2.5</v>
       </c>
       <c r="M166" t="n">
         <v>87.08</v>
       </c>
       <c r="N166" t="n">
-        <v>67.59999999999999</v>
+        <v>62.1</v>
       </c>
       <c r="O166" t="inlineStr">
         <is>
@@ -10277,7 +10053,7 @@
         </is>
       </c>
       <c r="P166" t="n">
-        <v>1</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="167">
@@ -10306,30 +10082,30 @@
         <v>3</v>
       </c>
       <c r="G167" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>The Resdev Scholar (IRE)</t>
+          <t>First Legion (IRE)</t>
         </is>
       </c>
       <c r="I167" t="n">
         <v>3</v>
       </c>
       <c r="J167" t="n">
-        <v>118</v>
+        <v>130</v>
       </c>
       <c r="K167" t="n">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="L167" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M167" t="n">
         <v>87.08</v>
       </c>
       <c r="N167" t="n">
-        <v>58.9</v>
+        <v>66.3</v>
       </c>
       <c r="O167" t="inlineStr">
         <is>
@@ -10337,7 +10113,7 @@
         </is>
       </c>
       <c r="P167" t="n">
-        <v>-4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="168">
@@ -10366,30 +10142,30 @@
         <v>3</v>
       </c>
       <c r="G168" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>Gold Queen Kindly (IRE)</t>
+          <t>Hasbro Market (IRE)</t>
         </is>
       </c>
       <c r="I168" t="n">
         <v>3</v>
       </c>
       <c r="J168" t="n">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="K168" t="n">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="L168" t="n">
-        <v>2.5</v>
+        <v>3.75</v>
       </c>
       <c r="M168" t="n">
         <v>87.08</v>
       </c>
       <c r="N168" t="n">
-        <v>62.1</v>
+        <v>63.3</v>
       </c>
       <c r="O168" t="inlineStr">
         <is>
@@ -10397,7 +10173,7 @@
         </is>
       </c>
       <c r="P168" t="n">
-        <v>-2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="169">
@@ -10426,30 +10202,30 @@
         <v>3</v>
       </c>
       <c r="G169" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>First Legion (IRE)</t>
+          <t>Ellusive Butterfly (IRE)</t>
         </is>
       </c>
       <c r="I169" t="n">
         <v>3</v>
       </c>
       <c r="J169" t="n">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="K169" t="n">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="L169" t="n">
-        <v>3</v>
+        <v>3.9</v>
       </c>
       <c r="M169" t="n">
         <v>87.08</v>
       </c>
       <c r="N169" t="n">
-        <v>66.3</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="O169" t="inlineStr">
         <is>
@@ -10457,7 +10233,7 @@
         </is>
       </c>
       <c r="P169" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="170">
@@ -10486,30 +10262,30 @@
         <v>3</v>
       </c>
       <c r="G170" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>Hasbro Market (IRE)</t>
+          <t>Inishbeg (IRE)</t>
         </is>
       </c>
       <c r="I170" t="n">
         <v>3</v>
       </c>
       <c r="J170" t="n">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="K170" t="n">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="L170" t="n">
-        <v>3.75</v>
+        <v>5.4</v>
       </c>
       <c r="M170" t="n">
         <v>87.08</v>
       </c>
       <c r="N170" t="n">
-        <v>63.3</v>
+        <v>54.3</v>
       </c>
       <c r="O170" t="inlineStr">
         <is>
@@ -10517,7 +10293,7 @@
         </is>
       </c>
       <c r="P170" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="171">
@@ -10546,30 +10322,30 @@
         <v>3</v>
       </c>
       <c r="G171" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>Ellusive Butterfly (IRE)</t>
+          <t>Al Najashi</t>
         </is>
       </c>
       <c r="I171" t="n">
         <v>3</v>
       </c>
       <c r="J171" t="n">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="K171" t="n">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="L171" t="n">
-        <v>3.9</v>
+        <v>8.15</v>
       </c>
       <c r="M171" t="n">
         <v>87.08</v>
       </c>
       <c r="N171" t="n">
-        <v>66.59999999999999</v>
+        <v>54.5</v>
       </c>
       <c r="O171" t="inlineStr">
         <is>
@@ -10577,7 +10353,7 @@
         </is>
       </c>
       <c r="P171" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="172">
@@ -10606,30 +10382,30 @@
         <v>3</v>
       </c>
       <c r="G172" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>Inishbeg (IRE)</t>
+          <t>Luansobe</t>
         </is>
       </c>
       <c r="I172" t="n">
         <v>3</v>
       </c>
       <c r="J172" t="n">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="K172" t="n">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="L172" t="n">
-        <v>5.4</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="M172" t="n">
         <v>87.08</v>
       </c>
       <c r="N172" t="n">
-        <v>54.3</v>
+        <v>42</v>
       </c>
       <c r="O172" t="inlineStr">
         <is>
@@ -10637,7 +10413,7 @@
         </is>
       </c>
       <c r="P172" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="173">
@@ -10666,30 +10442,30 @@
         <v>3</v>
       </c>
       <c r="G173" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>Al Najashi</t>
+          <t>First Time (IRE)</t>
         </is>
       </c>
       <c r="I173" t="n">
         <v>3</v>
       </c>
       <c r="J173" t="n">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="K173" t="n">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="L173" t="n">
-        <v>8.15</v>
+        <v>10.05</v>
       </c>
       <c r="M173" t="n">
         <v>87.08</v>
       </c>
       <c r="N173" t="n">
-        <v>54.5</v>
+        <v>39.3</v>
       </c>
       <c r="O173" t="inlineStr">
         <is>
@@ -10697,7 +10473,7 @@
         </is>
       </c>
       <c r="P173" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="174">
@@ -10726,30 +10502,30 @@
         <v>3</v>
       </c>
       <c r="G174" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>Luansobe</t>
+          <t>Montague Menace</t>
         </is>
       </c>
       <c r="I174" t="n">
         <v>3</v>
       </c>
       <c r="J174" t="n">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K174" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="L174" t="n">
-        <v>8.300000000000001</v>
+        <v>12.05</v>
       </c>
       <c r="M174" t="n">
         <v>87.08</v>
       </c>
       <c r="N174" t="n">
-        <v>42</v>
+        <v>30.1</v>
       </c>
       <c r="O174" t="inlineStr">
         <is>
@@ -10786,30 +10562,30 @@
         <v>3</v>
       </c>
       <c r="G175" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>First Time (IRE)</t>
+          <t>Awraad (IRE)</t>
         </is>
       </c>
       <c r="I175" t="n">
         <v>3</v>
       </c>
       <c r="J175" t="n">
-        <v>126</v>
+        <v>115</v>
       </c>
       <c r="K175" t="n">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="L175" t="n">
-        <v>10.05</v>
+        <v>17.55</v>
       </c>
       <c r="M175" t="n">
         <v>87.08</v>
       </c>
       <c r="N175" t="n">
-        <v>39.3</v>
+        <v>10.3</v>
       </c>
       <c r="O175" t="inlineStr">
         <is>
@@ -10817,7 +10593,7 @@
         </is>
       </c>
       <c r="P175" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="176">
@@ -10846,38 +10622,38 @@
         <v>3</v>
       </c>
       <c r="G176" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>Montague Menace</t>
+          <t>Advance Twentyfive (FR)</t>
         </is>
       </c>
       <c r="I176" t="n">
         <v>3</v>
       </c>
       <c r="J176" t="n">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="K176" t="n">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="L176" t="n">
-        <v>12.05</v>
+        <v>20.3</v>
       </c>
       <c r="M176" t="n">
         <v>87.08</v>
       </c>
       <c r="N176" t="n">
-        <v>30.1</v>
+        <v>29.2</v>
       </c>
       <c r="O176" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>low</t>
         </is>
       </c>
       <c r="P176" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="177">
@@ -10905,40 +10681,24 @@
       <c r="F177" t="n">
         <v>3</v>
       </c>
-      <c r="G177" t="n">
-        <v>13</v>
-      </c>
+      <c r="G177" t="inlineStr"/>
       <c r="H177" t="inlineStr">
         <is>
-          <t>Awraad (IRE)</t>
-        </is>
-      </c>
-      <c r="I177" t="n">
-        <v>3</v>
-      </c>
-      <c r="J177" t="n">
-        <v>120</v>
-      </c>
-      <c r="K177" t="n">
-        <v>80</v>
-      </c>
-      <c r="L177" t="n">
-        <v>17.55</v>
-      </c>
-      <c r="M177" t="n">
-        <v>87.08</v>
-      </c>
-      <c r="N177" t="n">
-        <v>12.9</v>
-      </c>
+          <t>Passing Thought</t>
+        </is>
+      </c>
+      <c r="I177" t="inlineStr"/>
+      <c r="J177" t="inlineStr"/>
+      <c r="K177" t="inlineStr"/>
+      <c r="L177" t="inlineStr"/>
+      <c r="M177" t="inlineStr"/>
+      <c r="N177" t="inlineStr"/>
       <c r="O177" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="P177" t="n">
-        <v>-1</v>
-      </c>
+      <c r="P177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -10965,40 +10725,24 @@
       <c r="F178" t="n">
         <v>3</v>
       </c>
-      <c r="G178" t="n">
-        <v>14</v>
-      </c>
+      <c r="G178" t="inlineStr"/>
       <c r="H178" t="inlineStr">
         <is>
-          <t>Advance Twentyfive (FR)</t>
-        </is>
-      </c>
-      <c r="I178" t="n">
-        <v>3</v>
-      </c>
-      <c r="J178" t="n">
-        <v>124</v>
-      </c>
-      <c r="K178" t="n">
-        <v>84</v>
-      </c>
-      <c r="L178" t="n">
-        <v>20.3</v>
-      </c>
-      <c r="M178" t="n">
-        <v>87.08</v>
-      </c>
-      <c r="N178" t="n">
-        <v>29.2</v>
-      </c>
+          <t>Cotai Lights (IRE)</t>
+        </is>
+      </c>
+      <c r="I178" t="inlineStr"/>
+      <c r="J178" t="inlineStr"/>
+      <c r="K178" t="inlineStr"/>
+      <c r="L178" t="inlineStr"/>
+      <c r="M178" t="inlineStr"/>
+      <c r="N178" t="inlineStr"/>
       <c r="O178" t="inlineStr">
         <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="P178" t="n">
-        <v>1</v>
-      </c>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -11155,7 +10899,7 @@
         <v>6</v>
       </c>
       <c r="J181" t="n">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="K181" t="n">
         <v>79</v>
@@ -11167,7 +10911,7 @@
         <v>152.75</v>
       </c>
       <c r="N181" t="n">
-        <v>79.40000000000001</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="O181" t="inlineStr">
         <is>
@@ -11235,7 +10979,7 @@
         </is>
       </c>
       <c r="P182" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="183">
@@ -11275,7 +11019,7 @@
         <v>4</v>
       </c>
       <c r="J183" t="n">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="K183" t="n">
         <v>84</v>
@@ -11287,7 +11031,7 @@
         <v>152.75</v>
       </c>
       <c r="N183" t="n">
-        <v>74.40000000000001</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="O183" t="inlineStr">
         <is>
@@ -11295,7 +11039,7 @@
         </is>
       </c>
       <c r="P183" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="184">
@@ -11655,7 +11399,7 @@
         </is>
       </c>
       <c r="P189" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="190">
@@ -11695,7 +11439,7 @@
         <v>5</v>
       </c>
       <c r="J190" t="n">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="K190" t="n">
         <v>75</v>
@@ -11707,7 +11451,7 @@
         <v>152.75</v>
       </c>
       <c r="N190" t="n">
-        <v>61.9</v>
+        <v>58.8</v>
       </c>
       <c r="O190" t="inlineStr">
         <is>
@@ -11715,7 +11459,7 @@
         </is>
       </c>
       <c r="P190" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="191">

</xml_diff>